<commit_message>
chore: update BIG3 weekly report 2026-05-25
</commit_message>
<xml_diff>
--- a/data/BIG3_tracker.xlsx
+++ b/data/BIG3_tracker.xlsx
@@ -318,12 +318,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'ベンチプレス'!$A$130:$A$139</f>
+              <f>'ベンチプレス'!$A$137:$A$146</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'ベンチプレス'!$C$130:$C$139</f>
+              <f>'ベンチプレス'!$C$137:$C$146</f>
             </numRef>
           </val>
         </ser>
@@ -638,7 +638,7 @@
     <from>
       <col>8</col>
       <colOff>0</colOff>
-      <row>127</row>
+      <row>134</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -1018,7 +1018,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BIG3 週次トラッカー  （更新: 2026-05-18）</t>
+          <t>BIG3 週次トラッカー  （更新: 2026-05-25）</t>
         </is>
       </c>
     </row>
@@ -1052,14 +1052,14 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>88.09999999999999</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="C4" s="4" t="n">
         <v>80</v>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-23</t>
         </is>
       </c>
     </row>
@@ -1155,17 +1155,17 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>85.2</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>1560</v>
+        <v>4060</v>
       </c>
       <c r="D10" s="8" t="n"/>
       <c r="E10" s="8" t="n"/>
       <c r="F10" s="8" t="n"/>
       <c r="G10" s="8" t="n"/>
       <c r="H10" s="9" t="n">
-        <v>1560</v>
+        <v>4060</v>
       </c>
     </row>
     <row r="11">
@@ -1391,7 +1391,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H139"/>
+  <dimension ref="A1:H146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1451,7 +1451,7 @@
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B4" s="10" t="inlineStr">
@@ -1480,7 +1480,7 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -1509,7 +1509,7 @@
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
@@ -1538,7 +1538,7 @@
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
@@ -1555,19 +1555,19 @@
         <v>77.5</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>310</v>
+        <v>542.5</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>85.2</v>
+        <v>91.09999999999999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
@@ -1584,19 +1584,19 @@
         <v>77.5</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F8" s="11" t="n">
-        <v>155</v>
+        <v>465</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>81.40000000000001</v>
+        <v>89.09999999999999</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
@@ -1609,231 +1609,231 @@
           <t>ベンチプレス　（バーベル）</t>
         </is>
       </c>
-      <c r="D9" s="8" t="n">
-        <v>60</v>
+      <c r="D9" s="9" t="n">
+        <v>77.5</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="F9" s="8" t="n">
-        <v>300</v>
+        <v>6</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>465</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>67.5</v>
+        <v>89.09999999999999</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>W20</t>
+          <t>W21</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>Bench Press (Barbell)</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="n">
-        <v>20</v>
+          <t>ベンチプレス　（バーベル）</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>77.5</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>10</v>
-      </c>
-      <c r="F10" s="10" t="n">
-        <v>200</v>
+        <v>3</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>232.5</v>
       </c>
       <c r="G10" s="11" t="n">
-        <v>25</v>
+        <v>83.3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>W20</t>
+          <t>W21</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Bench Press (Barbell)</t>
+          <t>ベンチプレス　（バーベル）</t>
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>57.5</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>W20</t>
+          <t>W21</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>Bench Press (Barbell)</t>
+          <t>ベンチプレス　（バーベル）</t>
         </is>
       </c>
       <c r="D12" s="10" t="n">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>195</v>
+        <v>400</v>
       </c>
       <c r="G12" s="11" t="n">
-        <v>69.90000000000001</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>W20</t>
+          <t>W21</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Bench Press (Barbell)</t>
+          <t>ベンチプレス　（バーベル）</t>
         </is>
       </c>
       <c r="D13" s="8" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>525</v>
+        <v>195</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>88.09999999999999</v>
+        <v>69.90000000000001</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>W20</t>
+          <t>W21</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>Bench Press (Barbell)</t>
-        </is>
-      </c>
-      <c r="D14" s="10" t="n">
-        <v>75</v>
+          <t>ベンチプレス　（バーベル）</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>77.5</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="F14" s="10" t="n">
-        <v>450</v>
+        <v>4</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>310</v>
       </c>
       <c r="G14" s="11" t="n">
-        <v>86.2</v>
+        <v>85.2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>W20</t>
+          <t>W21</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Bench Press (Barbell)</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="n">
-        <v>75</v>
+          <t>ベンチプレス　（バーベル）</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>77.5</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="F15" s="8" t="n">
-        <v>375</v>
+        <v>2</v>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>155</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>84.40000000000001</v>
+        <v>81.40000000000001</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>W19</t>
+          <t>W21</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>Bench Press (Barbell)</t>
+          <t>ベンチプレス　（バーベル）</t>
         </is>
       </c>
       <c r="D16" s="10" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="E16" s="10" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F16" s="10" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="G16" s="11" t="n">
-        <v>25</v>
+        <v>67.5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>W19</t>
+          <t>W20</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
@@ -1842,27 +1842,27 @@
         </is>
       </c>
       <c r="D17" s="8" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>W19</t>
+          <t>W20</t>
         </is>
       </c>
       <c r="C18" s="10" t="inlineStr">
@@ -1871,27 +1871,27 @@
         </is>
       </c>
       <c r="D18" s="10" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="E18" s="10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F18" s="10" t="n">
         <v>300</v>
       </c>
       <c r="G18" s="11" t="n">
-        <v>67.5</v>
+        <v>57.5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>W19</t>
+          <t>W20</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
@@ -1900,27 +1900,27 @@
         </is>
       </c>
       <c r="D19" s="8" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>70</v>
+        <v>195</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>71.8</v>
+        <v>69.90000000000001</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>W19</t>
+          <t>W20</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
@@ -1928,28 +1928,28 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D20" s="11" t="n">
-        <v>72.5</v>
+      <c r="D20" s="10" t="n">
+        <v>75</v>
       </c>
       <c r="E20" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="F20" s="11" t="n">
-        <v>507.5</v>
+      <c r="F20" s="10" t="n">
+        <v>525</v>
       </c>
       <c r="G20" s="11" t="n">
-        <v>85.2</v>
+        <v>88.09999999999999</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>W19</t>
+          <t>W20</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
@@ -1957,28 +1957,28 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D21" s="9" t="n">
-        <v>72.5</v>
+      <c r="D21" s="8" t="n">
+        <v>75</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="F21" s="9" t="n">
-        <v>580</v>
+        <v>6</v>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>450</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>87</v>
+        <v>86.2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>W19</t>
+          <t>W20</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
@@ -1986,17 +1986,17 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D22" s="11" t="n">
-        <v>72.5</v>
+      <c r="D22" s="10" t="n">
+        <v>75</v>
       </c>
       <c r="E22" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="F22" s="11" t="n">
-        <v>435</v>
+        <v>5</v>
+      </c>
+      <c r="F22" s="10" t="n">
+        <v>375</v>
       </c>
       <c r="G22" s="11" t="n">
-        <v>83.40000000000001</v>
+        <v>84.40000000000001</v>
       </c>
     </row>
     <row r="23">
@@ -2015,23 +2015,23 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D23" s="9" t="n">
-        <v>62.5</v>
+      <c r="D23" s="8" t="n">
+        <v>20</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>12</v>
-      </c>
-      <c r="F23" s="9" t="n">
-        <v>750</v>
+        <v>10</v>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>200</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>81.2</v>
+        <v>25</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
@@ -2045,22 +2045,22 @@
         </is>
       </c>
       <c r="D24" s="10" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="E24" s="10" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F24" s="10" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="G24" s="11" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
@@ -2074,22 +2074,22 @@
         </is>
       </c>
       <c r="D25" s="8" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>60</v>
+        <v>67.5</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
@@ -2103,22 +2103,22 @@
         </is>
       </c>
       <c r="D26" s="10" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="E26" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F26" s="10" t="n">
-        <v>180</v>
+        <v>70</v>
       </c>
       <c r="G26" s="11" t="n">
-        <v>64.5</v>
+        <v>71.8</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
@@ -2131,23 +2131,23 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D27" s="8" t="n">
-        <v>70</v>
+      <c r="D27" s="9" t="n">
+        <v>72.5</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="F27" s="8" t="n">
-        <v>560</v>
+        <v>7</v>
+      </c>
+      <c r="F27" s="9" t="n">
+        <v>507.5</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>84</v>
+        <v>85.2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B28" s="10" t="inlineStr">
@@ -2160,23 +2160,23 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D28" s="10" t="n">
-        <v>70</v>
+      <c r="D28" s="11" t="n">
+        <v>72.5</v>
       </c>
       <c r="E28" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="F28" s="10" t="n">
-        <v>560</v>
+      <c r="F28" s="11" t="n">
+        <v>580</v>
       </c>
       <c r="G28" s="11" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
@@ -2189,23 +2189,23 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D29" s="8" t="n">
-        <v>70</v>
+      <c r="D29" s="9" t="n">
+        <v>72.5</v>
       </c>
       <c r="E29" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="F29" s="8" t="n">
-        <v>420</v>
+      <c r="F29" s="9" t="n">
+        <v>435</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>80.5</v>
+        <v>83.40000000000001</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="B30" s="10" t="inlineStr">
@@ -2218,17 +2218,17 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D30" s="10" t="n">
-        <v>80</v>
+      <c r="D30" s="11" t="n">
+        <v>62.5</v>
       </c>
       <c r="E30" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="F30" s="10" t="n">
-        <v>80</v>
+        <v>12</v>
+      </c>
+      <c r="F30" s="11" t="n">
+        <v>750</v>
       </c>
       <c r="G30" s="11" t="n">
-        <v>82</v>
+        <v>81.2</v>
       </c>
     </row>
     <row r="31">
@@ -2248,27 +2248,27 @@
         </is>
       </c>
       <c r="D31" s="8" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="E31" s="8" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F31" s="8" t="n">
-        <v>480</v>
+        <v>200</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>72</v>
+        <v>25</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>W18</t>
+          <t>W19</t>
         </is>
       </c>
       <c r="C32" s="10" t="inlineStr">
@@ -2277,27 +2277,27 @@
         </is>
       </c>
       <c r="D32" s="10" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="E32" s="10" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F32" s="10" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="G32" s="11" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>W18</t>
+          <t>W19</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
@@ -2306,27 +2306,27 @@
         </is>
       </c>
       <c r="D33" s="8" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="E33" s="8" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>400</v>
+        <v>180</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>50</v>
+        <v>64.5</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B34" s="10" t="inlineStr">
         <is>
-          <t>W18</t>
+          <t>W19</t>
         </is>
       </c>
       <c r="C34" s="10" t="inlineStr">
@@ -2335,27 +2335,27 @@
         </is>
       </c>
       <c r="D34" s="10" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E34" s="10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F34" s="10" t="n">
-        <v>350</v>
+        <v>560</v>
       </c>
       <c r="G34" s="11" t="n">
-        <v>58.8</v>
+        <v>84</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>W18</t>
+          <t>W19</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
@@ -2364,27 +2364,27 @@
         </is>
       </c>
       <c r="D35" s="8" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="E35" s="8" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>60</v>
+        <v>560</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>61.5</v>
+        <v>84</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="10" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B36" s="10" t="inlineStr">
         <is>
-          <t>W18</t>
+          <t>W19</t>
         </is>
       </c>
       <c r="C36" s="10" t="inlineStr">
@@ -2393,27 +2393,27 @@
         </is>
       </c>
       <c r="D36" s="10" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="E36" s="10" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F36" s="10" t="n">
-        <v>65</v>
+        <v>420</v>
       </c>
       <c r="G36" s="11" t="n">
-        <v>66.59999999999999</v>
+        <v>80.5</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>W18</t>
+          <t>W19</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
@@ -2422,27 +2422,27 @@
         </is>
       </c>
       <c r="D37" s="8" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="E37" s="8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F37" s="8" t="n">
-        <v>350</v>
+        <v>80</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>78.8</v>
+        <v>82</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>W18</t>
+          <t>W19</t>
         </is>
       </c>
       <c r="C38" s="10" t="inlineStr">
@@ -2451,16 +2451,16 @@
         </is>
       </c>
       <c r="D38" s="10" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="E38" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F38" s="10" t="n">
-        <v>420</v>
+        <v>480</v>
       </c>
       <c r="G38" s="11" t="n">
-        <v>80.5</v>
+        <v>72</v>
       </c>
     </row>
     <row r="39">
@@ -2480,16 +2480,16 @@
         </is>
       </c>
       <c r="D39" s="8" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="E39" s="8" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>75.2</v>
+        <v>25</v>
       </c>
     </row>
     <row r="40">
@@ -2509,16 +2509,16 @@
         </is>
       </c>
       <c r="D40" s="10" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="E40" s="10" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F40" s="10" t="n">
-        <v>280</v>
+        <v>400</v>
       </c>
       <c r="G40" s="11" t="n">
-        <v>77</v>
+        <v>50</v>
       </c>
     </row>
     <row r="41">
@@ -2541,19 +2541,19 @@
         <v>50</v>
       </c>
       <c r="E41" s="8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F41" s="8" t="n">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="G41" s="9" t="n">
-        <v>57.5</v>
+        <v>58.8</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="10" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B42" s="10" t="inlineStr">
@@ -2567,22 +2567,22 @@
         </is>
       </c>
       <c r="D42" s="10" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="E42" s="10" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F42" s="10" t="n">
-        <v>200</v>
+        <v>60</v>
       </c>
       <c r="G42" s="11" t="n">
-        <v>25</v>
+        <v>61.5</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
@@ -2596,22 +2596,22 @@
         </is>
       </c>
       <c r="D43" s="8" t="n">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="E43" s="8" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F43" s="8" t="n">
-        <v>320</v>
+        <v>65</v>
       </c>
       <c r="G43" s="9" t="n">
-        <v>48</v>
+        <v>66.59999999999999</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B44" s="10" t="inlineStr">
@@ -2625,22 +2625,22 @@
         </is>
       </c>
       <c r="D44" s="10" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E44" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F44" s="10" t="n">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="G44" s="11" t="n">
-        <v>57.5</v>
+        <v>78.8</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
@@ -2654,22 +2654,22 @@
         </is>
       </c>
       <c r="D45" s="8" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="E45" s="8" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F45" s="8" t="n">
-        <v>60</v>
+        <v>420</v>
       </c>
       <c r="G45" s="9" t="n">
-        <v>61.5</v>
+        <v>80.5</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="10" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B46" s="10" t="inlineStr">
@@ -2682,23 +2682,23 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D46" s="11" t="n">
-        <v>67.5</v>
+      <c r="D46" s="10" t="n">
+        <v>70</v>
       </c>
       <c r="E46" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="F46" s="11" t="n">
-        <v>337.5</v>
+        <v>3</v>
+      </c>
+      <c r="F46" s="10" t="n">
+        <v>210</v>
       </c>
       <c r="G46" s="11" t="n">
-        <v>75.90000000000001</v>
+        <v>75.2</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="8" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B47" s="8" t="inlineStr">
@@ -2711,23 +2711,23 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D47" s="9" t="n">
-        <v>67.5</v>
+      <c r="D47" s="8" t="n">
+        <v>70</v>
       </c>
       <c r="E47" s="8" t="n">
-        <v>7</v>
-      </c>
-      <c r="F47" s="9" t="n">
-        <v>472.5</v>
+        <v>4</v>
+      </c>
+      <c r="F47" s="8" t="n">
+        <v>280</v>
       </c>
       <c r="G47" s="9" t="n">
-        <v>79.3</v>
+        <v>77</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="10" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B48" s="10" t="inlineStr">
@@ -2740,17 +2740,17 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D48" s="11" t="n">
-        <v>67.5</v>
+      <c r="D48" s="10" t="n">
+        <v>50</v>
       </c>
       <c r="E48" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="F48" s="11" t="n">
-        <v>270</v>
+        <v>6</v>
+      </c>
+      <c r="F48" s="10" t="n">
+        <v>300</v>
       </c>
       <c r="G48" s="11" t="n">
-        <v>74.2</v>
+        <v>57.5</v>
       </c>
     </row>
     <row r="49">
@@ -2769,17 +2769,17 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D49" s="9" t="n">
-        <v>67.5</v>
+      <c r="D49" s="8" t="n">
+        <v>20</v>
       </c>
       <c r="E49" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="F49" s="9" t="n">
-        <v>202.5</v>
+        <v>10</v>
+      </c>
+      <c r="F49" s="8" t="n">
+        <v>200</v>
       </c>
       <c r="G49" s="9" t="n">
-        <v>72.59999999999999</v>
+        <v>25</v>
       </c>
     </row>
     <row r="50">
@@ -2798,17 +2798,17 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D50" s="11" t="n">
-        <v>77.5</v>
+      <c r="D50" s="10" t="n">
+        <v>40</v>
       </c>
       <c r="E50" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="F50" s="11" t="n">
-        <v>77.5</v>
+        <v>8</v>
+      </c>
+      <c r="F50" s="10" t="n">
+        <v>320</v>
       </c>
       <c r="G50" s="11" t="n">
-        <v>79.40000000000001</v>
+        <v>48</v>
       </c>
     </row>
     <row r="51">
@@ -2828,27 +2828,27 @@
         </is>
       </c>
       <c r="D51" s="8" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="E51" s="8" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F51" s="8" t="n">
-        <v>480</v>
+        <v>300</v>
       </c>
       <c r="G51" s="9" t="n">
-        <v>72</v>
+        <v>57.5</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="10" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>W17</t>
+          <t>W18</t>
         </is>
       </c>
       <c r="C52" s="10" t="inlineStr">
@@ -2857,27 +2857,27 @@
         </is>
       </c>
       <c r="D52" s="10" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="E52" s="10" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F52" s="10" t="n">
-        <v>200</v>
+        <v>60</v>
       </c>
       <c r="G52" s="11" t="n">
-        <v>25</v>
+        <v>61.5</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>W17</t>
+          <t>W18</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
@@ -2885,28 +2885,28 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D53" s="8" t="n">
-        <v>40</v>
+      <c r="D53" s="9" t="n">
+        <v>67.5</v>
       </c>
       <c r="E53" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="F53" s="8" t="n">
-        <v>400</v>
+        <v>5</v>
+      </c>
+      <c r="F53" s="9" t="n">
+        <v>337.5</v>
       </c>
       <c r="G53" s="9" t="n">
-        <v>50</v>
+        <v>75.90000000000001</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="10" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B54" s="10" t="inlineStr">
         <is>
-          <t>W17</t>
+          <t>W18</t>
         </is>
       </c>
       <c r="C54" s="10" t="inlineStr">
@@ -2914,28 +2914,28 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D54" s="10" t="n">
-        <v>50</v>
+      <c r="D54" s="11" t="n">
+        <v>67.5</v>
       </c>
       <c r="E54" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="F54" s="10" t="n">
-        <v>250</v>
+        <v>7</v>
+      </c>
+      <c r="F54" s="11" t="n">
+        <v>472.5</v>
       </c>
       <c r="G54" s="11" t="n">
-        <v>56.2</v>
+        <v>79.3</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>W17</t>
+          <t>W18</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
@@ -2943,28 +2943,28 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D55" s="8" t="n">
-        <v>65</v>
+      <c r="D55" s="9" t="n">
+        <v>67.5</v>
       </c>
       <c r="E55" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="F55" s="8" t="n">
-        <v>195</v>
+        <v>4</v>
+      </c>
+      <c r="F55" s="9" t="n">
+        <v>270</v>
       </c>
       <c r="G55" s="9" t="n">
-        <v>69.90000000000001</v>
+        <v>74.2</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B56" s="10" t="inlineStr">
         <is>
-          <t>W17</t>
+          <t>W18</t>
         </is>
       </c>
       <c r="C56" s="10" t="inlineStr">
@@ -2972,28 +2972,28 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D56" s="10" t="n">
-        <v>65</v>
+      <c r="D56" s="11" t="n">
+        <v>67.5</v>
       </c>
       <c r="E56" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="F56" s="10" t="n">
-        <v>520</v>
+        <v>3</v>
+      </c>
+      <c r="F56" s="11" t="n">
+        <v>202.5</v>
       </c>
       <c r="G56" s="11" t="n">
-        <v>78</v>
+        <v>72.59999999999999</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>W17</t>
+          <t>W18</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
@@ -3001,28 +3001,28 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D57" s="8" t="n">
-        <v>65</v>
+      <c r="D57" s="9" t="n">
+        <v>77.5</v>
       </c>
       <c r="E57" s="8" t="n">
-        <v>7</v>
-      </c>
-      <c r="F57" s="8" t="n">
-        <v>455</v>
+        <v>1</v>
+      </c>
+      <c r="F57" s="9" t="n">
+        <v>77.5</v>
       </c>
       <c r="G57" s="9" t="n">
-        <v>76.40000000000001</v>
+        <v>79.40000000000001</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="10" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-29</t>
         </is>
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>W17</t>
+          <t>W18</t>
         </is>
       </c>
       <c r="C58" s="10" t="inlineStr">
@@ -3031,16 +3031,16 @@
         </is>
       </c>
       <c r="D58" s="10" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="E58" s="10" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F58" s="10" t="n">
-        <v>195</v>
+        <v>480</v>
       </c>
       <c r="G58" s="11" t="n">
-        <v>69.90000000000001</v>
+        <v>72</v>
       </c>
     </row>
     <row r="59">
@@ -3060,16 +3060,16 @@
         </is>
       </c>
       <c r="D59" s="8" t="n">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="E59" s="8" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F59" s="8" t="n">
-        <v>325</v>
+        <v>200</v>
       </c>
       <c r="G59" s="9" t="n">
-        <v>73.09999999999999</v>
+        <v>25</v>
       </c>
     </row>
     <row r="60">
@@ -3089,16 +3089,16 @@
         </is>
       </c>
       <c r="D60" s="10" t="n">
-        <v>65</v>
+        <v>40</v>
       </c>
       <c r="E60" s="10" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F60" s="10" t="n">
-        <v>325</v>
+        <v>400</v>
       </c>
       <c r="G60" s="11" t="n">
-        <v>73.09999999999999</v>
+        <v>50</v>
       </c>
     </row>
     <row r="61">
@@ -3118,22 +3118,22 @@
         </is>
       </c>
       <c r="D61" s="8" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="E61" s="8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F61" s="8" t="n">
-        <v>75</v>
+        <v>250</v>
       </c>
       <c r="G61" s="9" t="n">
-        <v>76.90000000000001</v>
+        <v>56.2</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="10" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
@@ -3147,22 +3147,22 @@
         </is>
       </c>
       <c r="D62" s="10" t="n">
-        <v>28</v>
+        <v>65</v>
       </c>
       <c r="E62" s="10" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F62" s="10" t="n">
-        <v>280</v>
+        <v>195</v>
       </c>
       <c r="G62" s="11" t="n">
-        <v>35</v>
+        <v>69.90000000000001</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B63" s="8" t="inlineStr">
@@ -3176,22 +3176,22 @@
         </is>
       </c>
       <c r="D63" s="8" t="n">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="E63" s="8" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F63" s="8" t="n">
-        <v>400</v>
+        <v>520</v>
       </c>
       <c r="G63" s="9" t="n">
-        <v>50</v>
+        <v>78</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="10" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B64" s="10" t="inlineStr">
@@ -3205,22 +3205,22 @@
         </is>
       </c>
       <c r="D64" s="10" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="E64" s="10" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F64" s="10" t="n">
-        <v>150</v>
+        <v>455</v>
       </c>
       <c r="G64" s="11" t="n">
-        <v>53.8</v>
+        <v>76.40000000000001</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B65" s="8" t="inlineStr">
@@ -3233,23 +3233,23 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D65" s="9" t="n">
-        <v>62.5</v>
+      <c r="D65" s="8" t="n">
+        <v>65</v>
       </c>
       <c r="E65" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="F65" s="9" t="n">
-        <v>500</v>
+        <v>3</v>
+      </c>
+      <c r="F65" s="8" t="n">
+        <v>195</v>
       </c>
       <c r="G65" s="9" t="n">
-        <v>75</v>
+        <v>69.90000000000001</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="10" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B66" s="10" t="inlineStr">
@@ -3262,23 +3262,23 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D66" s="11" t="n">
-        <v>62.5</v>
+      <c r="D66" s="10" t="n">
+        <v>65</v>
       </c>
       <c r="E66" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="F66" s="11" t="n">
-        <v>437.5</v>
+        <v>5</v>
+      </c>
+      <c r="F66" s="10" t="n">
+        <v>325</v>
       </c>
       <c r="G66" s="11" t="n">
-        <v>73.40000000000001</v>
+        <v>73.09999999999999</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B67" s="8" t="inlineStr">
@@ -3291,23 +3291,23 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D67" s="9" t="n">
-        <v>62.5</v>
+      <c r="D67" s="8" t="n">
+        <v>65</v>
       </c>
       <c r="E67" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="F67" s="9" t="n">
-        <v>500</v>
+        <v>5</v>
+      </c>
+      <c r="F67" s="8" t="n">
+        <v>325</v>
       </c>
       <c r="G67" s="9" t="n">
-        <v>75</v>
+        <v>73.09999999999999</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="10" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-25</t>
         </is>
       </c>
       <c r="B68" s="10" t="inlineStr">
@@ -3320,17 +3320,17 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D68" s="11" t="n">
-        <v>62.5</v>
+      <c r="D68" s="10" t="n">
+        <v>75</v>
       </c>
       <c r="E68" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="F68" s="11" t="n">
-        <v>500</v>
+        <v>1</v>
+      </c>
+      <c r="F68" s="10" t="n">
+        <v>75</v>
       </c>
       <c r="G68" s="11" t="n">
-        <v>75</v>
+        <v>76.90000000000001</v>
       </c>
     </row>
     <row r="69">
@@ -3349,17 +3349,17 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D69" s="9" t="n">
-        <v>62.5</v>
+      <c r="D69" s="8" t="n">
+        <v>28</v>
       </c>
       <c r="E69" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="F69" s="9" t="n">
-        <v>187.5</v>
+        <v>10</v>
+      </c>
+      <c r="F69" s="8" t="n">
+        <v>280</v>
       </c>
       <c r="G69" s="9" t="n">
-        <v>67.2</v>
+        <v>35</v>
       </c>
     </row>
     <row r="70">
@@ -3378,144 +3378,144 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D70" s="11" t="n">
-        <v>72.2</v>
+      <c r="D70" s="10" t="n">
+        <v>40</v>
       </c>
       <c r="E70" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="F70" s="11" t="n">
-        <v>72.2</v>
+        <v>10</v>
+      </c>
+      <c r="F70" s="10" t="n">
+        <v>400</v>
       </c>
       <c r="G70" s="11" t="n">
-        <v>74</v>
+        <v>50</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B71" s="8" t="inlineStr">
         <is>
-          <t>W16</t>
+          <t>W17</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t>Bench Press (Smith Machine)</t>
+          <t>Bench Press (Barbell)</t>
         </is>
       </c>
       <c r="D71" s="8" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="E71" s="8" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F71" s="8" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="G71" s="9" t="n">
-        <v>12.5</v>
+        <v>53.8</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="10" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t>W16</t>
+          <t>W17</t>
         </is>
       </c>
       <c r="C72" s="10" t="inlineStr">
         <is>
-          <t>Bench Press (Smith Machine)</t>
-        </is>
-      </c>
-      <c r="D72" s="10" t="n">
-        <v>20</v>
+          <t>Bench Press (Barbell)</t>
+        </is>
+      </c>
+      <c r="D72" s="11" t="n">
+        <v>62.5</v>
       </c>
       <c r="E72" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="F72" s="10" t="n">
-        <v>100</v>
+        <v>8</v>
+      </c>
+      <c r="F72" s="11" t="n">
+        <v>500</v>
       </c>
       <c r="G72" s="11" t="n">
-        <v>22.5</v>
+        <v>75</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B73" s="8" t="inlineStr">
         <is>
-          <t>W16</t>
+          <t>W17</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t>Bench Press (Smith Machine)</t>
-        </is>
-      </c>
-      <c r="D73" s="8" t="n">
-        <v>40</v>
+          <t>Bench Press (Barbell)</t>
+        </is>
+      </c>
+      <c r="D73" s="9" t="n">
+        <v>62.5</v>
       </c>
       <c r="E73" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="F73" s="8" t="n">
-        <v>200</v>
+        <v>7</v>
+      </c>
+      <c r="F73" s="9" t="n">
+        <v>437.5</v>
       </c>
       <c r="G73" s="9" t="n">
-        <v>45</v>
+        <v>73.40000000000001</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="10" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B74" s="10" t="inlineStr">
         <is>
-          <t>W16</t>
+          <t>W17</t>
         </is>
       </c>
       <c r="C74" s="10" t="inlineStr">
         <is>
-          <t>Bench Press (Smith Machine)</t>
-        </is>
-      </c>
-      <c r="D74" s="10" t="n">
-        <v>50</v>
+          <t>Bench Press (Barbell)</t>
+        </is>
+      </c>
+      <c r="D74" s="11" t="n">
+        <v>62.5</v>
       </c>
       <c r="E74" s="10" t="n">
-        <v>3</v>
-      </c>
-      <c r="F74" s="10" t="n">
-        <v>150</v>
+        <v>8</v>
+      </c>
+      <c r="F74" s="11" t="n">
+        <v>500</v>
       </c>
       <c r="G74" s="11" t="n">
-        <v>53.8</v>
+        <v>75</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B75" s="8" t="inlineStr">
         <is>
-          <t>W15</t>
+          <t>W17</t>
         </is>
       </c>
       <c r="C75" s="8" t="inlineStr">
@@ -3523,28 +3523,28 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D75" s="8" t="n">
-        <v>20</v>
+      <c r="D75" s="9" t="n">
+        <v>62.5</v>
       </c>
       <c r="E75" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="F75" s="8" t="n">
-        <v>200</v>
+        <v>8</v>
+      </c>
+      <c r="F75" s="9" t="n">
+        <v>500</v>
       </c>
       <c r="G75" s="9" t="n">
-        <v>25</v>
+        <v>75</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="10" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B76" s="10" t="inlineStr">
         <is>
-          <t>W15</t>
+          <t>W17</t>
         </is>
       </c>
       <c r="C76" s="10" t="inlineStr">
@@ -3552,28 +3552,28 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D76" s="10" t="n">
-        <v>40</v>
+      <c r="D76" s="11" t="n">
+        <v>62.5</v>
       </c>
       <c r="E76" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="F76" s="10" t="n">
-        <v>320</v>
+        <v>3</v>
+      </c>
+      <c r="F76" s="11" t="n">
+        <v>187.5</v>
       </c>
       <c r="G76" s="11" t="n">
-        <v>48</v>
+        <v>67.2</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="8" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B77" s="8" t="inlineStr">
         <is>
-          <t>W15</t>
+          <t>W17</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
@@ -3581,133 +3581,133 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D77" s="8" t="n">
-        <v>50</v>
+      <c r="D77" s="9" t="n">
+        <v>72.2</v>
       </c>
       <c r="E77" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="F77" s="8" t="n">
-        <v>250</v>
+        <v>1</v>
+      </c>
+      <c r="F77" s="9" t="n">
+        <v>72.2</v>
       </c>
       <c r="G77" s="9" t="n">
-        <v>56.2</v>
+        <v>74</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="10" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B78" s="10" t="inlineStr">
         <is>
-          <t>W15</t>
+          <t>W16</t>
         </is>
       </c>
       <c r="C78" s="10" t="inlineStr">
         <is>
-          <t>Bench Press (Barbell)</t>
+          <t>Bench Press (Smith Machine)</t>
         </is>
       </c>
       <c r="D78" s="10" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="E78" s="10" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F78" s="10" t="n">
-        <v>480</v>
+        <v>100</v>
       </c>
       <c r="G78" s="11" t="n">
-        <v>72</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B79" s="8" t="inlineStr">
         <is>
-          <t>W15</t>
+          <t>W16</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t>Bench Press (Barbell)</t>
+          <t>Bench Press (Smith Machine)</t>
         </is>
       </c>
       <c r="D79" s="8" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="E79" s="8" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F79" s="8" t="n">
-        <v>480</v>
+        <v>100</v>
       </c>
       <c r="G79" s="9" t="n">
-        <v>72</v>
+        <v>22.5</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="10" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B80" s="10" t="inlineStr">
         <is>
-          <t>W15</t>
+          <t>W16</t>
         </is>
       </c>
       <c r="C80" s="10" t="inlineStr">
         <is>
-          <t>Bench Press (Barbell)</t>
+          <t>Bench Press (Smith Machine)</t>
         </is>
       </c>
       <c r="D80" s="10" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="E80" s="10" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F80" s="10" t="n">
-        <v>480</v>
+        <v>200</v>
       </c>
       <c r="G80" s="11" t="n">
-        <v>72</v>
+        <v>45</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B81" s="8" t="inlineStr">
         <is>
-          <t>W15</t>
+          <t>W16</t>
         </is>
       </c>
       <c r="C81" s="8" t="inlineStr">
         <is>
-          <t>Bench Press (Barbell)</t>
+          <t>Bench Press (Smith Machine)</t>
         </is>
       </c>
       <c r="D81" s="8" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="E81" s="8" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F81" s="8" t="n">
-        <v>480</v>
+        <v>150</v>
       </c>
       <c r="G81" s="9" t="n">
-        <v>72</v>
+        <v>53.8</v>
       </c>
     </row>
     <row r="82">
@@ -3727,16 +3727,16 @@
         </is>
       </c>
       <c r="D82" s="10" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="E82" s="10" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F82" s="10" t="n">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="G82" s="11" t="n">
-        <v>75.2</v>
+        <v>25</v>
       </c>
     </row>
     <row r="83">
@@ -3756,22 +3756,22 @@
         </is>
       </c>
       <c r="D83" s="8" t="n">
-        <v>70</v>
+        <v>40</v>
       </c>
       <c r="E83" s="8" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F83" s="8" t="n">
-        <v>70</v>
+        <v>320</v>
       </c>
       <c r="G83" s="9" t="n">
-        <v>71.8</v>
+        <v>48</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="10" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B84" s="10" t="inlineStr">
@@ -3785,22 +3785,22 @@
         </is>
       </c>
       <c r="D84" s="10" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="E84" s="10" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F84" s="10" t="n">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="G84" s="11" t="n">
-        <v>25</v>
+        <v>56.2</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="8" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B85" s="8" t="inlineStr">
@@ -3814,22 +3814,22 @@
         </is>
       </c>
       <c r="D85" s="8" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="E85" s="8" t="n">
         <v>8</v>
       </c>
       <c r="F85" s="8" t="n">
-        <v>320</v>
+        <v>480</v>
       </c>
       <c r="G85" s="9" t="n">
-        <v>48</v>
+        <v>72</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="10" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B86" s="10" t="inlineStr">
@@ -3843,22 +3843,22 @@
         </is>
       </c>
       <c r="D86" s="10" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="E86" s="10" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F86" s="10" t="n">
-        <v>250</v>
+        <v>480</v>
       </c>
       <c r="G86" s="11" t="n">
-        <v>56.2</v>
+        <v>72</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B87" s="8" t="inlineStr">
@@ -3875,24 +3875,24 @@
         <v>60</v>
       </c>
       <c r="E87" s="8" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F87" s="8" t="n">
-        <v>240</v>
+        <v>480</v>
       </c>
       <c r="G87" s="9" t="n">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="10" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B88" s="10" t="inlineStr">
         <is>
-          <t>W14</t>
+          <t>W15</t>
         </is>
       </c>
       <c r="C88" s="10" t="inlineStr">
@@ -3901,27 +3901,27 @@
         </is>
       </c>
       <c r="D88" s="10" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="E88" s="10" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F88" s="10" t="n">
-        <v>200</v>
+        <v>480</v>
       </c>
       <c r="G88" s="11" t="n">
-        <v>25</v>
+        <v>72</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B89" s="8" t="inlineStr">
         <is>
-          <t>W14</t>
+          <t>W15</t>
         </is>
       </c>
       <c r="C89" s="8" t="inlineStr">
@@ -3930,27 +3930,27 @@
         </is>
       </c>
       <c r="D89" s="8" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E89" s="8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F89" s="8" t="n">
-        <v>250</v>
+        <v>210</v>
       </c>
       <c r="G89" s="9" t="n">
-        <v>56.2</v>
+        <v>75.2</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="10" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B90" s="10" t="inlineStr">
         <is>
-          <t>W14</t>
+          <t>W15</t>
         </is>
       </c>
       <c r="C90" s="10" t="inlineStr">
@@ -3958,28 +3958,28 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D90" s="11" t="n">
-        <v>57.5</v>
+      <c r="D90" s="10" t="n">
+        <v>70</v>
       </c>
       <c r="E90" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="F90" s="11" t="n">
-        <v>345</v>
+        <v>1</v>
+      </c>
+      <c r="F90" s="10" t="n">
+        <v>70</v>
       </c>
       <c r="G90" s="11" t="n">
-        <v>66.09999999999999</v>
+        <v>71.8</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="8" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B91" s="8" t="inlineStr">
         <is>
-          <t>W14</t>
+          <t>W15</t>
         </is>
       </c>
       <c r="C91" s="8" t="inlineStr">
@@ -3987,28 +3987,28 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D91" s="9" t="n">
-        <v>57.5</v>
+      <c r="D91" s="8" t="n">
+        <v>20</v>
       </c>
       <c r="E91" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="F91" s="9" t="n">
-        <v>460</v>
+        <v>10</v>
+      </c>
+      <c r="F91" s="8" t="n">
+        <v>200</v>
       </c>
       <c r="G91" s="9" t="n">
-        <v>69</v>
+        <v>25</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="10" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B92" s="10" t="inlineStr">
         <is>
-          <t>W14</t>
+          <t>W15</t>
         </is>
       </c>
       <c r="C92" s="10" t="inlineStr">
@@ -4016,28 +4016,28 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D92" s="11" t="n">
-        <v>57.5</v>
+      <c r="D92" s="10" t="n">
+        <v>40</v>
       </c>
       <c r="E92" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="F92" s="11" t="n">
-        <v>345</v>
+        <v>8</v>
+      </c>
+      <c r="F92" s="10" t="n">
+        <v>320</v>
       </c>
       <c r="G92" s="11" t="n">
-        <v>66.09999999999999</v>
+        <v>48</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="8" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B93" s="8" t="inlineStr">
         <is>
-          <t>W14</t>
+          <t>W15</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr">
@@ -4045,28 +4045,28 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D93" s="9" t="n">
-        <v>67.5</v>
+      <c r="D93" s="8" t="n">
+        <v>50</v>
       </c>
       <c r="E93" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="F93" s="9" t="n">
-        <v>135</v>
+        <v>5</v>
+      </c>
+      <c r="F93" s="8" t="n">
+        <v>250</v>
       </c>
       <c r="G93" s="9" t="n">
-        <v>70.90000000000001</v>
+        <v>56.2</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="10" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B94" s="10" t="inlineStr">
         <is>
-          <t>W14</t>
+          <t>W15</t>
         </is>
       </c>
       <c r="C94" s="10" t="inlineStr">
@@ -4075,22 +4075,22 @@
         </is>
       </c>
       <c r="D94" s="10" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="E94" s="10" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="F94" s="10" t="n">
-        <v>200</v>
+        <v>240</v>
       </c>
       <c r="G94" s="11" t="n">
-        <v>25</v>
+        <v>66</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="8" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B95" s="8" t="inlineStr">
@@ -4104,22 +4104,22 @@
         </is>
       </c>
       <c r="D95" s="8" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E95" s="8" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F95" s="8" t="n">
-        <v>240</v>
+        <v>200</v>
       </c>
       <c r="G95" s="9" t="n">
-        <v>46</v>
+        <v>25</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="10" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B96" s="10" t="inlineStr">
@@ -4136,19 +4136,19 @@
         <v>50</v>
       </c>
       <c r="E96" s="10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F96" s="10" t="n">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="G96" s="11" t="n">
-        <v>53.8</v>
+        <v>56.2</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="8" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B97" s="8" t="inlineStr">
@@ -4161,23 +4161,23 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D97" s="8" t="n">
-        <v>55</v>
+      <c r="D97" s="9" t="n">
+        <v>57.5</v>
       </c>
       <c r="E97" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="F97" s="8" t="n">
-        <v>440</v>
+        <v>6</v>
+      </c>
+      <c r="F97" s="9" t="n">
+        <v>345</v>
       </c>
       <c r="G97" s="9" t="n">
-        <v>66</v>
+        <v>66.09999999999999</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="10" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B98" s="10" t="inlineStr">
@@ -4190,23 +4190,23 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D98" s="10" t="n">
-        <v>55</v>
+      <c r="D98" s="11" t="n">
+        <v>57.5</v>
       </c>
       <c r="E98" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="F98" s="10" t="n">
-        <v>440</v>
+      <c r="F98" s="11" t="n">
+        <v>460</v>
       </c>
       <c r="G98" s="11" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="8" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B99" s="8" t="inlineStr">
@@ -4219,23 +4219,23 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D99" s="8" t="n">
-        <v>55</v>
+      <c r="D99" s="9" t="n">
+        <v>57.5</v>
       </c>
       <c r="E99" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="F99" s="8" t="n">
-        <v>275</v>
+        <v>6</v>
+      </c>
+      <c r="F99" s="9" t="n">
+        <v>345</v>
       </c>
       <c r="G99" s="9" t="n">
-        <v>61.9</v>
+        <v>66.09999999999999</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="10" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B100" s="10" t="inlineStr">
@@ -4248,220 +4248,220 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D100" s="10" t="n">
-        <v>65</v>
+      <c r="D100" s="11" t="n">
+        <v>67.5</v>
       </c>
       <c r="E100" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="F100" s="10" t="n">
-        <v>65</v>
+        <v>2</v>
+      </c>
+      <c r="F100" s="11" t="n">
+        <v>135</v>
       </c>
       <c r="G100" s="11" t="n">
-        <v>66.59999999999999</v>
+        <v>70.90000000000001</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="8" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B101" s="8" t="inlineStr">
         <is>
-          <t>W13</t>
+          <t>W14</t>
         </is>
       </c>
       <c r="C101" s="8" t="inlineStr">
         <is>
-          <t>Bench Press (Smith Machine)</t>
+          <t>Bench Press (Barbell)</t>
         </is>
       </c>
       <c r="D101" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="E101" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="E101" s="8" t="n">
-        <v>5</v>
-      </c>
       <c r="F101" s="8" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="G101" s="9" t="n">
-        <v>11.2</v>
+        <v>25</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="10" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B102" s="10" t="inlineStr">
         <is>
-          <t>W13</t>
+          <t>W14</t>
         </is>
       </c>
       <c r="C102" s="10" t="inlineStr">
         <is>
-          <t>Bench Press (Smith Machine)</t>
+          <t>Bench Press (Barbell)</t>
         </is>
       </c>
       <c r="D102" s="10" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="E102" s="10" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F102" s="10" t="n">
         <v>240</v>
       </c>
       <c r="G102" s="11" t="n">
-        <v>36</v>
+        <v>46</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="8" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B103" s="8" t="inlineStr">
         <is>
-          <t>W13</t>
+          <t>W14</t>
         </is>
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t>Bench Press (Smith Machine)</t>
+          <t>Bench Press (Barbell)</t>
         </is>
       </c>
       <c r="D103" s="8" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="E103" s="8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F103" s="8" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="G103" s="9" t="n">
-        <v>45</v>
+        <v>53.8</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="10" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B104" s="10" t="inlineStr">
         <is>
-          <t>W13</t>
+          <t>W14</t>
         </is>
       </c>
       <c r="C104" s="10" t="inlineStr">
         <is>
-          <t>Bench Press (Smith Machine)</t>
+          <t>Bench Press (Barbell)</t>
         </is>
       </c>
       <c r="D104" s="10" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="E104" s="10" t="n">
         <v>8</v>
       </c>
       <c r="F104" s="10" t="n">
-        <v>400</v>
+        <v>440</v>
       </c>
       <c r="G104" s="11" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="8" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B105" s="8" t="inlineStr">
         <is>
-          <t>W13</t>
+          <t>W14</t>
         </is>
       </c>
       <c r="C105" s="8" t="inlineStr">
         <is>
-          <t>Bench Press (Smith Machine)</t>
+          <t>Bench Press (Barbell)</t>
         </is>
       </c>
       <c r="D105" s="8" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="E105" s="8" t="n">
         <v>8</v>
       </c>
       <c r="F105" s="8" t="n">
-        <v>400</v>
+        <v>440</v>
       </c>
       <c r="G105" s="9" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="10" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B106" s="10" t="inlineStr">
         <is>
-          <t>W13</t>
+          <t>W14</t>
         </is>
       </c>
       <c r="C106" s="10" t="inlineStr">
         <is>
-          <t>Bench Press (Smith Machine)</t>
+          <t>Bench Press (Barbell)</t>
         </is>
       </c>
       <c r="D106" s="10" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="E106" s="10" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F106" s="10" t="n">
-        <v>400</v>
+        <v>275</v>
       </c>
       <c r="G106" s="11" t="n">
-        <v>60</v>
+        <v>61.9</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="8" t="inlineStr">
         <is>
-          <t>2026-03-29</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B107" s="8" t="inlineStr">
         <is>
-          <t>W13</t>
+          <t>W14</t>
         </is>
       </c>
       <c r="C107" s="8" t="inlineStr">
         <is>
-          <t>Bench Press (Smith Machine)</t>
+          <t>Bench Press (Barbell)</t>
         </is>
       </c>
       <c r="D107" s="8" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="E107" s="8" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="F107" s="8" t="n">
-        <v>500</v>
+        <v>65</v>
       </c>
       <c r="G107" s="9" t="n">
-        <v>62.5</v>
+        <v>66.59999999999999</v>
       </c>
     </row>
     <row r="108">
@@ -4481,16 +4481,16 @@
         </is>
       </c>
       <c r="D108" s="10" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="E108" s="10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F108" s="10" t="n">
-        <v>360</v>
+        <v>50</v>
       </c>
       <c r="G108" s="11" t="n">
-        <v>69</v>
+        <v>11.2</v>
       </c>
     </row>
     <row r="109">
@@ -4510,16 +4510,16 @@
         </is>
       </c>
       <c r="D109" s="8" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="E109" s="8" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F109" s="8" t="n">
-        <v>300</v>
+        <v>240</v>
       </c>
       <c r="G109" s="9" t="n">
-        <v>67.5</v>
+        <v>36</v>
       </c>
     </row>
     <row r="110">
@@ -4542,19 +4542,19 @@
         <v>40</v>
       </c>
       <c r="E110" s="10" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F110" s="10" t="n">
-        <v>320</v>
+        <v>200</v>
       </c>
       <c r="G110" s="11" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="8" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B111" s="8" t="inlineStr">
@@ -4564,26 +4564,26 @@
       </c>
       <c r="C111" s="8" t="inlineStr">
         <is>
-          <t>Bench Press (Barbell)</t>
+          <t>Bench Press (Smith Machine)</t>
         </is>
       </c>
       <c r="D111" s="8" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="E111" s="8" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F111" s="8" t="n">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="G111" s="9" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="10" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B112" s="10" t="inlineStr">
@@ -4593,26 +4593,26 @@
       </c>
       <c r="C112" s="10" t="inlineStr">
         <is>
-          <t>Bench Press (Barbell)</t>
+          <t>Bench Press (Smith Machine)</t>
         </is>
       </c>
       <c r="D112" s="10" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="E112" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F112" s="10" t="n">
-        <v>240</v>
+        <v>400</v>
       </c>
       <c r="G112" s="11" t="n">
-        <v>46</v>
+        <v>60</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="8" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B113" s="8" t="inlineStr">
@@ -4622,26 +4622,26 @@
       </c>
       <c r="C113" s="8" t="inlineStr">
         <is>
-          <t>Bench Press (Barbell)</t>
+          <t>Bench Press (Smith Machine)</t>
         </is>
       </c>
       <c r="D113" s="8" t="n">
         <v>50</v>
       </c>
       <c r="E113" s="8" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F113" s="8" t="n">
-        <v>150</v>
+        <v>400</v>
       </c>
       <c r="G113" s="9" t="n">
-        <v>53.8</v>
+        <v>60</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="10" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B114" s="10" t="inlineStr">
@@ -4651,26 +4651,26 @@
       </c>
       <c r="C114" s="10" t="inlineStr">
         <is>
-          <t>Bench Press (Barbell)</t>
-        </is>
-      </c>
-      <c r="D114" s="11" t="n">
-        <v>52.5</v>
+          <t>Bench Press (Smith Machine)</t>
+        </is>
+      </c>
+      <c r="D114" s="10" t="n">
+        <v>50</v>
       </c>
       <c r="E114" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="F114" s="11" t="n">
-        <v>315</v>
+        <v>10</v>
+      </c>
+      <c r="F114" s="10" t="n">
+        <v>500</v>
       </c>
       <c r="G114" s="11" t="n">
-        <v>60.4</v>
+        <v>62.5</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="8" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B115" s="8" t="inlineStr">
@@ -4680,26 +4680,26 @@
       </c>
       <c r="C115" s="8" t="inlineStr">
         <is>
-          <t>Bench Press (Barbell)</t>
-        </is>
-      </c>
-      <c r="D115" s="9" t="n">
-        <v>52.5</v>
+          <t>Bench Press (Smith Machine)</t>
+        </is>
+      </c>
+      <c r="D115" s="8" t="n">
+        <v>60</v>
       </c>
       <c r="E115" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="F115" s="9" t="n">
-        <v>315</v>
+      <c r="F115" s="8" t="n">
+        <v>360</v>
       </c>
       <c r="G115" s="9" t="n">
-        <v>60.4</v>
+        <v>69</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="10" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B116" s="10" t="inlineStr">
@@ -4709,26 +4709,26 @@
       </c>
       <c r="C116" s="10" t="inlineStr">
         <is>
-          <t>Bench Press (Barbell)</t>
-        </is>
-      </c>
-      <c r="D116" s="11" t="n">
-        <v>52.5</v>
+          <t>Bench Press (Smith Machine)</t>
+        </is>
+      </c>
+      <c r="D116" s="10" t="n">
+        <v>60</v>
       </c>
       <c r="E116" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="F116" s="11" t="n">
-        <v>420</v>
+        <v>5</v>
+      </c>
+      <c r="F116" s="10" t="n">
+        <v>300</v>
       </c>
       <c r="G116" s="11" t="n">
-        <v>63</v>
+        <v>67.5</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="8" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-29</t>
         </is>
       </c>
       <c r="B117" s="8" t="inlineStr">
@@ -4738,20 +4738,20 @@
       </c>
       <c r="C117" s="8" t="inlineStr">
         <is>
-          <t>Bench Press (Barbell)</t>
-        </is>
-      </c>
-      <c r="D117" s="9" t="n">
-        <v>52.5</v>
+          <t>Bench Press (Smith Machine)</t>
+        </is>
+      </c>
+      <c r="D117" s="8" t="n">
+        <v>40</v>
       </c>
       <c r="E117" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="F117" s="9" t="n">
-        <v>420</v>
+      <c r="F117" s="8" t="n">
+        <v>320</v>
       </c>
       <c r="G117" s="9" t="n">
-        <v>63</v>
+        <v>48</v>
       </c>
     </row>
     <row r="118">
@@ -4770,17 +4770,17 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D118" s="11" t="n">
-        <v>52.5</v>
+      <c r="D118" s="10" t="n">
+        <v>20</v>
       </c>
       <c r="E118" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="F118" s="11" t="n">
-        <v>315</v>
+        <v>10</v>
+      </c>
+      <c r="F118" s="10" t="n">
+        <v>200</v>
       </c>
       <c r="G118" s="11" t="n">
-        <v>60.4</v>
+        <v>25</v>
       </c>
     </row>
     <row r="119">
@@ -4799,28 +4799,28 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D119" s="9" t="n">
-        <v>62.5</v>
+      <c r="D119" s="8" t="n">
+        <v>40</v>
       </c>
       <c r="E119" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="F119" s="9" t="n">
-        <v>125</v>
+        <v>6</v>
+      </c>
+      <c r="F119" s="8" t="n">
+        <v>240</v>
       </c>
       <c r="G119" s="9" t="n">
-        <v>65.59999999999999</v>
+        <v>46</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="10" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B120" s="10" t="inlineStr">
         <is>
-          <t>W12</t>
+          <t>W13</t>
         </is>
       </c>
       <c r="C120" s="10" t="inlineStr">
@@ -4829,27 +4829,27 @@
         </is>
       </c>
       <c r="D120" s="10" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="E120" s="10" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F120" s="10" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="G120" s="11" t="n">
-        <v>25</v>
+        <v>53.8</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="8" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B121" s="8" t="inlineStr">
         <is>
-          <t>W12</t>
+          <t>W13</t>
         </is>
       </c>
       <c r="C121" s="8" t="inlineStr">
@@ -4857,28 +4857,28 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D121" s="8" t="n">
-        <v>40</v>
+      <c r="D121" s="9" t="n">
+        <v>52.5</v>
       </c>
       <c r="E121" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="F121" s="8" t="n">
-        <v>320</v>
+        <v>6</v>
+      </c>
+      <c r="F121" s="9" t="n">
+        <v>315</v>
       </c>
       <c r="G121" s="9" t="n">
-        <v>48</v>
+        <v>60.4</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="10" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B122" s="10" t="inlineStr">
         <is>
-          <t>W12</t>
+          <t>W13</t>
         </is>
       </c>
       <c r="C122" s="10" t="inlineStr">
@@ -4886,28 +4886,28 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D122" s="10" t="n">
-        <v>50</v>
+      <c r="D122" s="11" t="n">
+        <v>52.5</v>
       </c>
       <c r="E122" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="F122" s="10" t="n">
-        <v>400</v>
+        <v>6</v>
+      </c>
+      <c r="F122" s="11" t="n">
+        <v>315</v>
       </c>
       <c r="G122" s="11" t="n">
-        <v>60</v>
+        <v>60.4</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="8" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B123" s="8" t="inlineStr">
         <is>
-          <t>W12</t>
+          <t>W13</t>
         </is>
       </c>
       <c r="C123" s="8" t="inlineStr">
@@ -4915,28 +4915,28 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D123" s="8" t="n">
-        <v>50</v>
+      <c r="D123" s="9" t="n">
+        <v>52.5</v>
       </c>
       <c r="E123" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="F123" s="8" t="n">
-        <v>400</v>
+      <c r="F123" s="9" t="n">
+        <v>420</v>
       </c>
       <c r="G123" s="9" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="10" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B124" s="10" t="inlineStr">
         <is>
-          <t>W12</t>
+          <t>W13</t>
         </is>
       </c>
       <c r="C124" s="10" t="inlineStr">
@@ -4944,28 +4944,28 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D124" s="10" t="n">
-        <v>50</v>
+      <c r="D124" s="11" t="n">
+        <v>52.5</v>
       </c>
       <c r="E124" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="F124" s="10" t="n">
-        <v>300</v>
+        <v>8</v>
+      </c>
+      <c r="F124" s="11" t="n">
+        <v>420</v>
       </c>
       <c r="G124" s="11" t="n">
-        <v>57.5</v>
+        <v>63</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="8" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B125" s="8" t="inlineStr">
         <is>
-          <t>W12</t>
+          <t>W13</t>
         </is>
       </c>
       <c r="C125" s="8" t="inlineStr">
@@ -4973,310 +4973,513 @@
           <t>Bench Press (Barbell)</t>
         </is>
       </c>
-      <c r="D125" s="8" t="n">
-        <v>50</v>
+      <c r="D125" s="9" t="n">
+        <v>52.5</v>
       </c>
       <c r="E125" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="F125" s="8" t="n">
-        <v>400</v>
+        <v>6</v>
+      </c>
+      <c r="F125" s="9" t="n">
+        <v>315</v>
       </c>
       <c r="G125" s="9" t="n">
-        <v>60</v>
+        <v>60.4</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="10" t="inlineStr">
         <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B126" s="10" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="C126" s="10" t="inlineStr">
+        <is>
+          <t>Bench Press (Barbell)</t>
+        </is>
+      </c>
+      <c r="D126" s="11" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="E126" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F126" s="11" t="n">
+        <v>125</v>
+      </c>
+      <c r="G126" s="11" t="n">
+        <v>65.59999999999999</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="8" t="inlineStr">
+        <is>
           <t>2026-03-19</t>
         </is>
       </c>
-      <c r="B126" s="10" t="inlineStr">
+      <c r="B127" s="8" t="inlineStr">
         <is>
           <t>W12</t>
         </is>
       </c>
-      <c r="C126" s="10" t="inlineStr">
-        <is>
-          <t>Bench Press (Barbell)</t>
-        </is>
-      </c>
-      <c r="D126" s="10" t="n">
+      <c r="C127" s="8" t="inlineStr">
+        <is>
+          <t>Bench Press (Barbell)</t>
+        </is>
+      </c>
+      <c r="D127" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="E127" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="F127" s="8" t="n">
+        <v>200</v>
+      </c>
+      <c r="G127" s="9" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="10" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B128" s="10" t="inlineStr">
+        <is>
+          <t>W12</t>
+        </is>
+      </c>
+      <c r="C128" s="10" t="inlineStr">
+        <is>
+          <t>Bench Press (Barbell)</t>
+        </is>
+      </c>
+      <c r="D128" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="E128" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="F128" s="10" t="n">
+        <v>320</v>
+      </c>
+      <c r="G128" s="11" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B129" s="8" t="inlineStr">
+        <is>
+          <t>W12</t>
+        </is>
+      </c>
+      <c r="C129" s="8" t="inlineStr">
+        <is>
+          <t>Bench Press (Barbell)</t>
+        </is>
+      </c>
+      <c r="D129" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="E129" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="F129" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="G129" s="9" t="n">
         <v>60</v>
       </c>
-      <c r="E126" s="10" t="n">
+    </row>
+    <row r="130">
+      <c r="A130" s="10" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B130" s="10" t="inlineStr">
+        <is>
+          <t>W12</t>
+        </is>
+      </c>
+      <c r="C130" s="10" t="inlineStr">
+        <is>
+          <t>Bench Press (Barbell)</t>
+        </is>
+      </c>
+      <c r="D130" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="E130" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="F130" s="10" t="n">
+        <v>400</v>
+      </c>
+      <c r="G130" s="11" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B131" s="8" t="inlineStr">
+        <is>
+          <t>W12</t>
+        </is>
+      </c>
+      <c r="C131" s="8" t="inlineStr">
+        <is>
+          <t>Bench Press (Barbell)</t>
+        </is>
+      </c>
+      <c r="D131" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="E131" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="F131" s="8" t="n">
+        <v>300</v>
+      </c>
+      <c r="G131" s="9" t="n">
+        <v>57.5</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="10" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B132" s="10" t="inlineStr">
+        <is>
+          <t>W12</t>
+        </is>
+      </c>
+      <c r="C132" s="10" t="inlineStr">
+        <is>
+          <t>Bench Press (Barbell)</t>
+        </is>
+      </c>
+      <c r="D132" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="E132" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="F132" s="10" t="n">
+        <v>400</v>
+      </c>
+      <c r="G132" s="11" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="8" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B133" s="8" t="inlineStr">
+        <is>
+          <t>W12</t>
+        </is>
+      </c>
+      <c r="C133" s="8" t="inlineStr">
+        <is>
+          <t>Bench Press (Barbell)</t>
+        </is>
+      </c>
+      <c r="D133" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="E133" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="F126" s="10" t="n">
+      <c r="F133" s="8" t="n">
         <v>180</v>
       </c>
-      <c r="G126" s="11" t="n">
+      <c r="G133" s="9" t="n">
         <v>64.5</v>
       </c>
     </row>
-    <row r="128" ht="22" customHeight="1">
-      <c r="A128" s="13" t="inlineStr">
+    <row r="135" ht="22" customHeight="1">
+      <c r="A135" s="13" t="inlineStr">
         <is>
           <t>週別集計</t>
         </is>
       </c>
     </row>
-    <row r="129">
-      <c r="A129" s="2" t="inlineStr">
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
         <is>
           <t>週</t>
         </is>
       </c>
-      <c r="B129" s="2" t="inlineStr">
+      <c r="B136" s="2" t="inlineStr">
         <is>
           <t>最大重量 (kg)</t>
         </is>
       </c>
-      <c r="C129" s="2" t="inlineStr">
+      <c r="C136" s="2" t="inlineStr">
         <is>
           <t>推定1RM (kg)</t>
         </is>
       </c>
-      <c r="D129" s="2" t="inlineStr">
+      <c r="D136" s="2" t="inlineStr">
         <is>
           <t>総Volume (kg)</t>
         </is>
       </c>
-      <c r="E129" s="2" t="inlineStr">
+      <c r="E136" s="2" t="inlineStr">
         <is>
           <t>セッション数</t>
         </is>
       </c>
-      <c r="F129" s="2" t="inlineStr">
+      <c r="F136" s="2" t="inlineStr">
         <is>
           <t>セット数</t>
         </is>
       </c>
     </row>
-    <row r="130">
-      <c r="A130" s="8" t="inlineStr">
+    <row r="137">
+      <c r="A137" s="8" t="inlineStr">
         <is>
           <t>2026-W12</t>
         </is>
       </c>
-      <c r="B130" s="8" t="n">
+      <c r="B137" s="8" t="n">
         <v>60</v>
       </c>
-      <c r="C130" s="9" t="n">
+      <c r="C137" s="9" t="n">
         <v>64.5</v>
       </c>
-      <c r="D130" s="9" t="n">
+      <c r="D137" s="9" t="n">
         <v>2200</v>
       </c>
-      <c r="E130" s="8" t="n">
+      <c r="E137" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="F130" s="8" t="n">
+      <c r="F137" s="8" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="131">
-      <c r="A131" s="10" t="inlineStr">
+    <row r="138">
+      <c r="A138" s="10" t="inlineStr">
         <is>
           <t>2026-W13</t>
         </is>
       </c>
-      <c r="B131" s="11" t="n">
+      <c r="B138" s="11" t="n">
         <v>62.5</v>
       </c>
-      <c r="C131" s="11" t="n">
+      <c r="C138" s="11" t="n">
         <v>69</v>
       </c>
-      <c r="D131" s="11" t="n">
+      <c r="D138" s="11" t="n">
         <v>5670</v>
       </c>
-      <c r="E131" s="10" t="n">
+      <c r="E138" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F131" s="10" t="n">
+      <c r="F138" s="10" t="n">
         <v>19</v>
       </c>
     </row>
-    <row r="132">
-      <c r="A132" s="8" t="inlineStr">
+    <row r="139">
+      <c r="A139" s="8" t="inlineStr">
         <is>
           <t>2026-W14</t>
         </is>
       </c>
-      <c r="B132" s="9" t="n">
+      <c r="B139" s="9" t="n">
         <v>67.5</v>
       </c>
-      <c r="C132" s="9" t="n">
+      <c r="C139" s="9" t="n">
         <v>70.90000000000001</v>
       </c>
-      <c r="D132" s="9" t="n">
+      <c r="D139" s="9" t="n">
         <v>3545</v>
       </c>
-      <c r="E132" s="8" t="n">
+      <c r="E139" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="F132" s="8" t="n">
+      <c r="F139" s="8" t="n">
         <v>13</v>
       </c>
     </row>
-    <row r="133">
-      <c r="A133" s="10" t="inlineStr">
+    <row r="140">
+      <c r="A140" s="10" t="inlineStr">
         <is>
           <t>2026-W15</t>
         </is>
       </c>
-      <c r="B133" s="10" t="n">
+      <c r="B140" s="10" t="n">
         <v>70</v>
       </c>
-      <c r="C133" s="11" t="n">
+      <c r="C140" s="11" t="n">
         <v>75.2</v>
       </c>
-      <c r="D133" s="11" t="n">
+      <c r="D140" s="11" t="n">
         <v>3980</v>
       </c>
-      <c r="E133" s="10" t="n">
+      <c r="E140" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F133" s="10" t="n">
+      <c r="F140" s="10" t="n">
         <v>13</v>
       </c>
     </row>
-    <row r="134">
-      <c r="A134" s="8" t="inlineStr">
+    <row r="141">
+      <c r="A141" s="8" t="inlineStr">
         <is>
           <t>2026-W16</t>
         </is>
       </c>
-      <c r="B134" s="8" t="n">
+      <c r="B141" s="8" t="n">
         <v>50</v>
       </c>
-      <c r="C134" s="9" t="n">
+      <c r="C141" s="9" t="n">
         <v>53.8</v>
       </c>
-      <c r="D134" s="9" t="n">
+      <c r="D141" s="9" t="n">
         <v>550</v>
       </c>
-      <c r="E134" s="8" t="n">
+      <c r="E141" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="F134" s="8" t="n">
+      <c r="F141" s="8" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="135">
-      <c r="A135" s="10" t="inlineStr">
+    <row r="142">
+      <c r="A142" s="10" t="inlineStr">
         <is>
           <t>2026-W17</t>
         </is>
       </c>
-      <c r="B135" s="10" t="n">
+      <c r="B142" s="10" t="n">
         <v>75</v>
       </c>
-      <c r="C135" s="11" t="n">
+      <c r="C142" s="11" t="n">
         <v>78</v>
       </c>
-      <c r="D135" s="11" t="n">
+      <c r="D142" s="11" t="n">
         <v>5967.2</v>
       </c>
-      <c r="E135" s="10" t="n">
+      <c r="E142" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F135" s="10" t="n">
+      <c r="F142" s="10" t="n">
         <v>19</v>
       </c>
     </row>
-    <row r="136">
-      <c r="A136" s="8" t="inlineStr">
+    <row r="143">
+      <c r="A143" s="8" t="inlineStr">
         <is>
           <t>2026-W18</t>
         </is>
       </c>
-      <c r="B136" s="9" t="n">
+      <c r="B143" s="9" t="n">
         <v>77.5</v>
       </c>
-      <c r="C136" s="9" t="n">
+      <c r="C143" s="9" t="n">
         <v>80.5</v>
       </c>
-      <c r="D136" s="9" t="n">
+      <c r="D143" s="9" t="n">
         <v>5355</v>
       </c>
-      <c r="E136" s="8" t="n">
+      <c r="E143" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="F136" s="8" t="n">
+      <c r="F143" s="8" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="137">
-      <c r="A137" s="10" t="inlineStr">
+    <row r="144">
+      <c r="A144" s="10" t="inlineStr">
         <is>
           <t>2026-W19</t>
         </is>
       </c>
-      <c r="B137" s="10" t="n">
+      <c r="B144" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="C137" s="11" t="n">
+      <c r="C144" s="11" t="n">
         <v>87</v>
       </c>
-      <c r="D137" s="11" t="n">
+      <c r="D144" s="11" t="n">
         <v>6122.5</v>
       </c>
-      <c r="E137" s="10" t="n">
+      <c r="E144" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F137" s="10" t="n">
+      <c r="F144" s="10" t="n">
         <v>16</v>
       </c>
     </row>
-    <row r="138">
-      <c r="A138" s="8" t="inlineStr">
+    <row r="145">
+      <c r="A145" s="8" t="inlineStr">
         <is>
           <t>2026-W20</t>
         </is>
       </c>
-      <c r="B138" s="8" t="n">
+      <c r="B145" s="8" t="n">
         <v>75</v>
       </c>
-      <c r="C138" s="9" t="n">
+      <c r="C145" s="9" t="n">
         <v>88.09999999999999</v>
       </c>
-      <c r="D138" s="9" t="n">
+      <c r="D145" s="9" t="n">
         <v>2045</v>
       </c>
-      <c r="E138" s="8" t="n">
+      <c r="E145" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="F138" s="8" t="n">
+      <c r="F145" s="8" t="n">
         <v>6</v>
       </c>
     </row>
-    <row r="139">
-      <c r="A139" s="10" t="inlineStr">
+    <row r="146">
+      <c r="A146" s="10" t="inlineStr">
         <is>
           <t>2026-W21</t>
         </is>
       </c>
-      <c r="B139" s="11" t="n">
+      <c r="B146" s="11" t="n">
         <v>77.5</v>
       </c>
-      <c r="C139" s="11" t="n">
-        <v>85.2</v>
-      </c>
-      <c r="D139" s="11" t="n">
-        <v>1560</v>
-      </c>
-      <c r="E139" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="F139" s="10" t="n">
-        <v>6</v>
+      <c r="C146" s="11" t="n">
+        <v>91.09999999999999</v>
+      </c>
+      <c r="D146" s="11" t="n">
+        <v>4060</v>
+      </c>
+      <c r="E146" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F146" s="10" t="n">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A128:G128"/>
+    <mergeCell ref="A135:G135"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>